<commit_message>
fix webinar tracking, persistent scheduler, academy link, report command
</commit_message>
<xml_diff>
--- a/analytics_aptechka.xlsx
+++ b/analytics_aptechka.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>19.06.2026 02:26</t>
+          <t>19.06.2026 09:17</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -791,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -831,11 +831,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>19.06.2026 01:15</t>
+          <t>19.06.2026 10:58</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>291461984</v>
+        <v>1273451178</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -856,11 +856,11 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>19.06.2026 01:15</t>
+          <t>19.06.2026 09:17</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>291461984</v>
+        <v>1273451178</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
@@ -881,7 +881,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>19.06.2026 01:14</t>
+          <t>19.06.2026 09:17</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -894,7 +894,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>webinar_offered</t>
+          <t>bot_started</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -906,7 +906,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>19.06.2026 01:14</t>
+          <t>19.06.2026 03:33</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
@@ -931,7 +931,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>19.06.2026 00:36</t>
+          <t>19.06.2026 03:33</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -944,7 +944,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>bot_started</t>
+          <t>webinar_offered</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -956,7 +956,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>19.06.2026 00:36</t>
+          <t>19.06.2026 02:26</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
@@ -989,7 +989,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>дорогая мама</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -997,54 +997,66 @@
           <t>bot_started</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>19.06.2026 02:26</t>
+          <t>19.06.2026 01:15</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>1273451178</v>
+        <v>291461984</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>дорогая мама</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>webinar_offered</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr"/>
+          <t>bot_started</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>19.06.2026 03:33</t>
+          <t>19.06.2026 01:15</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>1273451178</v>
+        <v>291461984</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>дорогая мама</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>bot_started</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
+          <t>webinar_offered</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>19.06.2026 03:33</t>
+          <t>19.06.2026 01:14</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
@@ -1052,15 +1064,115 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>webinar_offered</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>19.06.2026 01:14</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>1273451178</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>bot_started</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>19.06.2026 00:36</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>1273451178</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>bot_started</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>19.06.2026 00:36</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>1273451178</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>webinar_offered</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>19.06.2026 10:59</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>1273451178</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
           <t>дорогая мама</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>webinar_offered</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>